<commit_message>
Actualización de prompts de mensajes para el corredor.
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B618FD-5BD2-411F-8F1C-5B201334EF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1DDE92-3CFA-41E8-9B40-2CB257C944DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -523,7 +523,7 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>3925178</xdr:colOff>
       <xdr:row>69</xdr:row>
-      <xdr:rowOff>80203</xdr:rowOff>
+      <xdr:rowOff>80202</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1242,7 +1242,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>22</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>46250</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>23</v>
       </c>
@@ -1569,7 +1569,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G27" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:G29" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">
       <filters blank="1">
         <filter val="Pendiente"/>

</xml_diff>

<commit_message>
Mejoras en el dashboard
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1DDE92-3CFA-41E8-9B40-2CB257C944DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0286F970-CDCF-420B-B473-7B3160299F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="61">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -323,12 +323,18 @@
   <si>
     <t>Crear end point para llamar y enviar mensajes del saldo y las notas de crédito</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/live/h0WhYGR7pdA?t=523s - Dejar de trabajar a los 57</t>
+  </si>
+  <si>
+    <t>Investigar como automatizar cosas con Power Automate</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -354,6 +360,14 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -414,10 +428,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -445,8 +460,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1508,6 +1527,16 @@
         <v>58</v>
       </c>
     </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C30" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="51" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E51">
         <v>28401.05</v>
@@ -1576,8 +1605,11 @@
       </filters>
     </filterColumn>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="C31" r:id="rId1" xr:uid="{3C22A885-07EB-43DB-A866-EAD7FAA5DC07}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>